<commit_message>
Sync review data 2026-10-22
</commit_message>
<xml_diff>
--- a/review-results/复盘信息抓取-20261022.xlsx
+++ b/review-results/复盘信息抓取-20261022.xlsx
@@ -1125,13 +1125,29 @@
           <t>00:15</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n"/>
+      <c r="D2" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E2" s="3" t="n">
         <v>296.95</v>
       </c>
       <c r="I2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S2" s="3" t="n"/>
       <c r="T2" s="3" t="n"/>
     </row>
@@ -1149,13 +1165,29 @@
           <t>00:30</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
+      <c r="D3" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E3" s="3" t="n">
         <v>380.55</v>
       </c>
       <c r="I3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S3" s="3" t="n"/>
       <c r="T3" s="3" t="n"/>
     </row>
@@ -1173,13 +1205,29 @@
           <t>00:45</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
+      <c r="D4" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E4" s="3" t="n">
         <v>296.95</v>
       </c>
       <c r="I4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S4" s="3" t="n"/>
       <c r="T4" s="3" t="n"/>
     </row>
@@ -1197,14 +1245,30 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n"/>
+      <c r="D5" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E5" s="3" t="n">
         <v>293.73</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
+      <c r="L5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
     </row>
@@ -1222,14 +1286,30 @@
           <t>01:15</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n"/>
+      <c r="D6" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E6" s="3" t="n">
         <v>380.73</v>
       </c>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
+      <c r="L6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S6" s="3" t="n"/>
       <c r="T6" s="3" t="n"/>
     </row>
@@ -1247,14 +1327,30 @@
           <t>01:30</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n"/>
+      <c r="D7" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E7" s="3" t="n">
         <v>292.19</v>
       </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
+      <c r="L7" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S7" s="3" t="n"/>
       <c r="T7" s="3" t="n"/>
     </row>
@@ -1272,14 +1368,30 @@
           <t>01:45</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n"/>
+      <c r="D8" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E8" s="3" t="n">
         <v>290</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
+      <c r="L8" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>01:45</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S8" s="3" t="n"/>
       <c r="T8" s="3" t="n"/>
     </row>
@@ -1297,14 +1409,30 @@
           <t>02:00</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n"/>
+      <c r="D9" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E9" s="3" t="n">
         <v>297.44</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
+      <c r="L9" t="n">
+        <v>8</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S9" s="3" t="n"/>
       <c r="T9" s="3" t="n"/>
     </row>
@@ -1322,14 +1450,30 @@
           <t>02:15</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n"/>
+      <c r="D10" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E10" s="3" t="n">
         <v>193.66</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="L10" t="n">
+        <v>9</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S10" s="3" t="n"/>
       <c r="T10" s="3" t="n"/>
     </row>
@@ -1347,14 +1491,30 @@
           <t>02:30</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n"/>
+      <c r="D11" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E11" s="3" t="n">
         <v>435.35</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
+      <c r="L11" t="n">
+        <v>10</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S11" s="3" t="n"/>
       <c r="T11" s="3" t="n"/>
     </row>
@@ -1372,14 +1532,30 @@
           <t>02:45</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n"/>
+      <c r="D12" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E12" s="3" t="n">
         <v>316.98</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
+      <c r="L12" t="n">
+        <v>11</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S12" s="3" t="n"/>
       <c r="T12" s="3" t="n"/>
     </row>
@@ -1397,14 +1573,30 @@
           <t>03:00</t>
         </is>
       </c>
-      <c r="D13" s="3" t="n"/>
+      <c r="D13" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E13" s="3" t="n">
         <v>180.11</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
+      <c r="L13" t="n">
+        <v>12</v>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S13" s="3" t="n"/>
       <c r="T13" s="3" t="n"/>
     </row>
@@ -1422,13 +1614,29 @@
           <t>03:15</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n"/>
+      <c r="D14" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E14" s="3" t="n">
         <v>184.36</v>
       </c>
       <c r="I14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
+      <c r="L14" t="n">
+        <v>13</v>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S14" s="3" t="n"/>
       <c r="T14" s="3" t="n"/>
     </row>
@@ -1446,13 +1654,29 @@
           <t>03:30</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n"/>
+      <c r="D15" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E15" s="3" t="n">
         <v>184.61</v>
       </c>
       <c r="I15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
+      <c r="L15" t="n">
+        <v>14</v>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="n"/>
     </row>
@@ -1470,13 +1694,29 @@
           <t>03:45</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n"/>
+      <c r="D16" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E16" s="3" t="n">
         <v>146</v>
       </c>
       <c r="I16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
+      <c r="L16" t="n">
+        <v>15</v>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S16" s="3" t="n"/>
       <c r="T16" s="3" t="n"/>
     </row>
@@ -1494,13 +1734,29 @@
           <t>04:00</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n"/>
+      <c r="D17" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E17" s="3" t="n">
         <v>144.8</v>
       </c>
       <c r="I17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="O17" s="3" t="n"/>
+      <c r="L17" t="n">
+        <v>16</v>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S17" s="3" t="n"/>
       <c r="T17" s="3" t="n"/>
     </row>
@@ -1518,13 +1774,29 @@
           <t>04:15</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n"/>
+      <c r="D18" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E18" s="3" t="n">
         <v>189.64</v>
       </c>
       <c r="I18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
+      <c r="L18" t="n">
+        <v>17</v>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S18" s="3" t="n"/>
       <c r="T18" s="3" t="n"/>
     </row>
@@ -1542,14 +1814,30 @@
           <t>04:30</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n"/>
+      <c r="D19" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E19" s="3" t="n">
         <v>184.61</v>
       </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="O19" s="3" t="n"/>
+      <c r="L19" t="n">
+        <v>18</v>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S19" s="3" t="n"/>
       <c r="T19" s="3" t="n"/>
     </row>
@@ -1567,14 +1855,30 @@
           <t>04:45</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n"/>
+      <c r="D20" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E20" s="3" t="n">
         <v>189.64</v>
       </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="O20" s="3" t="n"/>
+      <c r="L20" t="n">
+        <v>19</v>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S20" s="3" t="n"/>
       <c r="T20" s="3" t="n"/>
     </row>
@@ -1592,14 +1896,30 @@
           <t>05:00</t>
         </is>
       </c>
-      <c r="D21" s="3" t="n"/>
+      <c r="D21" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E21" s="3" t="n">
         <v>293.73</v>
       </c>
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
+      <c r="L21" t="n">
+        <v>20</v>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>445.32</v>
+      </c>
       <c r="S21" s="3" t="n"/>
       <c r="T21" s="3" t="n"/>
     </row>
@@ -1617,14 +1937,30 @@
           <t>05:15</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n"/>
+      <c r="D22" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E22" s="3" t="n">
         <v>294.1</v>
       </c>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
+      <c r="L22" t="n">
+        <v>21</v>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S22" s="3" t="n"/>
       <c r="T22" s="3" t="n"/>
     </row>
@@ -1642,14 +1978,30 @@
           <t>05:30</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n"/>
+      <c r="D23" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E23" s="3" t="n">
         <v>297.44</v>
       </c>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
+      <c r="L23" t="n">
+        <v>22</v>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S23" s="3" t="n"/>
       <c r="T23" s="3" t="n"/>
     </row>
@@ -1667,14 +2019,30 @@
           <t>05:45</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n"/>
+      <c r="D24" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E24" s="3" t="n">
         <v>350.04</v>
       </c>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
+      <c r="L24" t="n">
+        <v>23</v>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S24" s="3" t="n"/>
       <c r="T24" s="3" t="n"/>
     </row>
@@ -1692,14 +2060,30 @@
           <t>06:00</t>
         </is>
       </c>
-      <c r="D25" s="3" t="n"/>
+      <c r="D25" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E25" s="3" t="n">
         <v>300.57</v>
       </c>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="O25" s="3" t="n"/>
+      <c r="L25" t="n">
+        <v>24</v>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
     </row>
@@ -1717,14 +2101,30 @@
           <t>06:15</t>
         </is>
       </c>
-      <c r="D26" s="3" t="n"/>
+      <c r="D26" s="3" t="n">
+        <v>153.77</v>
+      </c>
       <c r="E26" s="3" t="n">
         <v>435.35</v>
       </c>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
+      <c r="L26" t="n">
+        <v>25</v>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S26" s="3" t="n"/>
       <c r="T26" s="3" t="n"/>
     </row>
@@ -1742,14 +2142,30 @@
           <t>06:30</t>
         </is>
       </c>
-      <c r="D27" s="3" t="n"/>
+      <c r="D27" s="3" t="n">
+        <v>153.77</v>
+      </c>
       <c r="E27" s="3" t="n">
         <v>453.33</v>
       </c>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
+      <c r="L27" t="n">
+        <v>26</v>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S27" s="3" t="n"/>
       <c r="T27" s="3" t="n"/>
     </row>
@@ -1767,14 +2183,30 @@
           <t>06:45</t>
         </is>
       </c>
-      <c r="D28" s="3" t="n"/>
+      <c r="D28" s="3" t="n">
+        <v>153.77</v>
+      </c>
       <c r="E28" s="3" t="n">
         <v>466.7</v>
       </c>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
+      <c r="L28" t="n">
+        <v>27</v>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S28" s="3" t="n"/>
       <c r="T28" s="3" t="n"/>
     </row>
@@ -1792,14 +2224,30 @@
           <t>07:00</t>
         </is>
       </c>
-      <c r="D29" s="3" t="n"/>
+      <c r="D29" s="3" t="n">
+        <v>153.77</v>
+      </c>
       <c r="E29" s="3" t="n">
         <v>466.55</v>
       </c>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="O29" s="3" t="n"/>
+      <c r="L29" t="n">
+        <v>28</v>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S29" s="3" t="n"/>
       <c r="T29" s="3" t="n"/>
     </row>
@@ -1817,14 +2265,30 @@
           <t>07:15</t>
         </is>
       </c>
-      <c r="D30" s="3" t="n"/>
+      <c r="D30" s="3" t="n">
+        <v>181.69</v>
+      </c>
       <c r="E30" s="3" t="n">
         <v>452.22</v>
       </c>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
+      <c r="L30" t="n">
+        <v>29</v>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>468.29</v>
+      </c>
       <c r="S30" s="3" t="n"/>
       <c r="T30" s="3" t="n"/>
     </row>
@@ -1842,14 +2306,30 @@
           <t>07:30</t>
         </is>
       </c>
-      <c r="D31" s="3" t="n"/>
+      <c r="D31" s="3" t="n">
+        <v>181.69</v>
+      </c>
       <c r="E31" s="3" t="n">
         <v>370</v>
       </c>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="O31" s="3" t="n"/>
+      <c r="L31" t="n">
+        <v>30</v>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>468.29</v>
+      </c>
       <c r="S31" s="3" t="n"/>
       <c r="T31" s="3" t="n"/>
     </row>
@@ -1867,14 +2347,30 @@
           <t>07:45</t>
         </is>
       </c>
-      <c r="D32" s="3" t="n"/>
+      <c r="D32" s="3" t="n">
+        <v>181.69</v>
+      </c>
       <c r="E32" s="3" t="n">
         <v>144.07</v>
       </c>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="O32" s="3" t="n"/>
+      <c r="L32" t="n">
+        <v>31</v>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>468.29</v>
+      </c>
       <c r="S32" s="3" t="n"/>
       <c r="T32" s="3" t="n"/>
     </row>
@@ -1892,14 +2388,30 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="D33" s="3" t="n"/>
+      <c r="D33" s="3" t="n">
+        <v>181.69</v>
+      </c>
       <c r="E33" s="3" t="n">
         <v>133.88</v>
       </c>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
-      <c r="M33" s="3" t="n"/>
-      <c r="O33" s="3" t="n"/>
+      <c r="L33" t="n">
+        <v>32</v>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>466.64</v>
+      </c>
       <c r="S33" s="3" t="n"/>
       <c r="T33" s="3" t="n"/>
     </row>
@@ -1917,14 +2429,30 @@
           <t>08:15</t>
         </is>
       </c>
-      <c r="D34" s="3" t="n"/>
+      <c r="D34" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E34" s="3" t="n">
         <v>133.88</v>
       </c>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
-      <c r="O34" s="3" t="n"/>
+      <c r="L34" t="n">
+        <v>33</v>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S34" s="3" t="n"/>
       <c r="T34" s="3" t="n"/>
     </row>
@@ -1942,14 +2470,30 @@
           <t>08:30</t>
         </is>
       </c>
-      <c r="D35" s="3" t="n"/>
+      <c r="D35" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E35" s="3" t="n">
         <v>107.54</v>
       </c>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="O35" s="3" t="n"/>
+      <c r="L35" t="n">
+        <v>34</v>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>220.14</v>
+      </c>
       <c r="S35" s="3" t="n"/>
       <c r="T35" s="3" t="n"/>
     </row>
@@ -1967,14 +2511,30 @@
           <t>08:45</t>
         </is>
       </c>
-      <c r="D36" s="3" t="n"/>
+      <c r="D36" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
-      <c r="M36" s="3" t="n"/>
-      <c r="O36" s="3" t="n"/>
+      <c r="L36" t="n">
+        <v>35</v>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>220.14</v>
+      </c>
       <c r="S36" s="3" t="n"/>
       <c r="T36" s="3" t="n"/>
     </row>
@@ -1992,14 +2552,30 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D37" s="3" t="n"/>
+      <c r="D37" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
-      <c r="M37" s="3" t="n"/>
-      <c r="O37" s="3" t="n"/>
+      <c r="L37" t="n">
+        <v>36</v>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>220.14</v>
+      </c>
       <c r="S37" s="3" t="n"/>
       <c r="T37" s="3" t="n"/>
     </row>
@@ -2017,14 +2593,30 @@
           <t>09:15</t>
         </is>
       </c>
-      <c r="D38" s="3" t="n"/>
+      <c r="D38" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E38" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="O38" s="3" t="n"/>
+      <c r="L38" t="n">
+        <v>37</v>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S38" s="3" t="n"/>
       <c r="T38" s="3" t="n"/>
     </row>
@@ -2042,14 +2634,30 @@
           <t>09:30</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n"/>
+      <c r="D39" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
+      <c r="L39" t="n">
+        <v>38</v>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S39" s="3" t="n"/>
       <c r="T39" s="3" t="n"/>
     </row>
@@ -2067,14 +2675,30 @@
           <t>09:45</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n"/>
+      <c r="D40" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E40" s="3" t="n">
         <v>133.88</v>
       </c>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
-      <c r="M40" s="3" t="n"/>
-      <c r="O40" s="3" t="n"/>
+      <c r="L40" t="n">
+        <v>39</v>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S40" s="3" t="n"/>
       <c r="T40" s="3" t="n"/>
     </row>
@@ -2092,14 +2716,30 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n"/>
+      <c r="D41" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E41" s="3" t="n">
         <v>460</v>
       </c>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
-      <c r="M41" s="3" t="n"/>
-      <c r="O41" s="3" t="n"/>
+      <c r="L41" t="n">
+        <v>40</v>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="n"/>
     </row>
@@ -2117,14 +2757,30 @@
           <t>10:15</t>
         </is>
       </c>
-      <c r="D42" s="3" t="n"/>
+      <c r="D42" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E42" s="3" t="n">
         <v>193.66</v>
       </c>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
-      <c r="M42" s="3" t="n"/>
-      <c r="O42" s="3" t="n"/>
+      <c r="L42" t="n">
+        <v>41</v>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S42" s="3" t="n"/>
       <c r="T42" s="3" t="n"/>
     </row>
@@ -2142,14 +2798,30 @@
           <t>10:30</t>
         </is>
       </c>
-      <c r="D43" s="3" t="n"/>
+      <c r="D43" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E43" s="3" t="n">
         <v>133.88</v>
       </c>
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
-      <c r="M43" s="3" t="n"/>
-      <c r="O43" s="3" t="n"/>
+      <c r="L43" t="n">
+        <v>42</v>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S43" s="3" t="n"/>
       <c r="T43" s="3" t="n"/>
     </row>
@@ -2167,14 +2839,30 @@
           <t>10:45</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n"/>
+      <c r="D44" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E44" s="3" t="n">
         <v>143.97</v>
       </c>
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
-      <c r="M44" s="3" t="n"/>
-      <c r="O44" s="3" t="n"/>
+      <c r="L44" t="n">
+        <v>43</v>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S44" s="3" t="n"/>
       <c r="T44" s="3" t="n"/>
     </row>
@@ -2192,14 +2880,30 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="D45" s="3" t="n"/>
+      <c r="D45" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E45" s="3" t="n">
         <v>153.77</v>
       </c>
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
-      <c r="M45" s="3" t="n"/>
-      <c r="O45" s="3" t="n"/>
+      <c r="L45" t="n">
+        <v>44</v>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S45" s="3" t="n"/>
       <c r="T45" s="3" t="n"/>
     </row>
@@ -2217,14 +2921,30 @@
           <t>11:15</t>
         </is>
       </c>
-      <c r="D46" s="3" t="n"/>
+      <c r="D46" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E46" s="3" t="n">
         <v>180.11</v>
       </c>
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
-      <c r="M46" s="3" t="n"/>
-      <c r="O46" s="3" t="n"/>
+      <c r="L46" t="n">
+        <v>45</v>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S46" s="3" t="n"/>
       <c r="T46" s="3" t="n"/>
     </row>
@@ -2242,14 +2962,30 @@
           <t>11:30</t>
         </is>
       </c>
-      <c r="D47" s="3" t="n"/>
+      <c r="D47" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E47" s="3" t="n">
         <v>293.76</v>
       </c>
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
-      <c r="M47" s="3" t="n"/>
-      <c r="O47" s="3" t="n"/>
+      <c r="L47" t="n">
+        <v>46</v>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="O47" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S47" s="3" t="n"/>
       <c r="T47" s="3" t="n"/>
     </row>
@@ -2267,14 +3003,30 @@
           <t>11:45</t>
         </is>
       </c>
-      <c r="D48" s="3" t="n"/>
+      <c r="D48" s="3" t="n">
+        <v>140.75</v>
+      </c>
       <c r="E48" s="3" t="n">
         <v>300.48</v>
       </c>
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
-      <c r="M48" s="3" t="n"/>
-      <c r="O48" s="3" t="n"/>
+      <c r="L48" t="n">
+        <v>47</v>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S48" s="3" t="n"/>
       <c r="T48" s="3" t="n"/>
     </row>
@@ -2292,14 +3044,30 @@
           <t>12:00</t>
         </is>
       </c>
-      <c r="D49" s="3" t="n"/>
+      <c r="D49" s="3" t="n">
+        <v>153.77</v>
+      </c>
       <c r="E49" s="3" t="n">
         <v>106.93</v>
       </c>
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
-      <c r="M49" s="3" t="n"/>
-      <c r="O49" s="3" t="n"/>
+      <c r="L49" t="n">
+        <v>48</v>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S49" s="3" t="n"/>
       <c r="T49" s="3" t="n"/>
     </row>
@@ -2317,14 +3085,30 @@
           <t>12:15</t>
         </is>
       </c>
-      <c r="D50" s="3" t="n"/>
+      <c r="D50" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E50" s="3" t="n">
         <v>106.93</v>
       </c>
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
-      <c r="M50" s="3" t="n"/>
-      <c r="O50" s="3" t="n"/>
+      <c r="L50" t="n">
+        <v>49</v>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="O50" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S50" s="3" t="n"/>
       <c r="T50" s="3" t="n"/>
     </row>
@@ -2342,14 +3126,30 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D51" s="3" t="n"/>
+      <c r="D51" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E51" s="3" t="n">
         <v>290.55</v>
       </c>
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
-      <c r="M51" s="3" t="n"/>
-      <c r="O51" s="3" t="n"/>
+      <c r="L51" t="n">
+        <v>50</v>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S51" s="3" t="n"/>
       <c r="T51" s="3" t="n"/>
     </row>
@@ -2367,14 +3167,30 @@
           <t>12:45</t>
         </is>
       </c>
-      <c r="D52" s="3" t="n"/>
+      <c r="D52" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E52" s="3" t="n">
         <v>133.69</v>
       </c>
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
-      <c r="M52" s="3" t="n"/>
-      <c r="O52" s="3" t="n"/>
+      <c r="L52" t="n">
+        <v>51</v>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S52" s="3" t="n"/>
       <c r="T52" s="3" t="n"/>
     </row>
@@ -2392,14 +3208,30 @@
           <t>13:00</t>
         </is>
       </c>
-      <c r="D53" s="3" t="n"/>
+      <c r="D53" s="3" t="n">
+        <v>181.69</v>
+      </c>
       <c r="E53" s="3" t="n">
         <v>316.98</v>
       </c>
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
-      <c r="M53" s="3" t="n"/>
-      <c r="O53" s="3" t="n"/>
+      <c r="L53" t="n">
+        <v>52</v>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S53" s="3" t="n"/>
       <c r="T53" s="3" t="n"/>
     </row>
@@ -2417,14 +3249,30 @@
           <t>13:15</t>
         </is>
       </c>
-      <c r="D54" s="3" t="n"/>
+      <c r="D54" s="3" t="n">
+        <v>247.64</v>
+      </c>
       <c r="E54" s="3" t="n">
         <v>180.11</v>
       </c>
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
-      <c r="M54" s="3" t="n"/>
-      <c r="O54" s="3" t="n"/>
+      <c r="L54" t="n">
+        <v>53</v>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="O54" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S54" s="3" t="n"/>
       <c r="T54" s="3" t="n"/>
     </row>
@@ -2442,14 +3290,30 @@
           <t>13:30</t>
         </is>
       </c>
-      <c r="D55" s="3" t="n"/>
+      <c r="D55" s="3" t="n">
+        <v>263.48</v>
+      </c>
       <c r="E55" s="3" t="n">
         <v>452.22</v>
       </c>
       <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
-      <c r="M55" s="3" t="n"/>
-      <c r="O55" s="3" t="n"/>
+      <c r="L55" t="n">
+        <v>54</v>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="O55" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="S55" s="3" t="n"/>
       <c r="T55" s="3" t="n"/>
     </row>
@@ -2467,14 +3331,30 @@
           <t>13:45</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n"/>
+      <c r="D56" s="3" t="n">
+        <v>247.64</v>
+      </c>
       <c r="E56" s="3" t="n">
         <v>464.92</v>
       </c>
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
-      <c r="M56" s="3" t="n"/>
-      <c r="O56" s="3" t="n"/>
+      <c r="L56" t="n">
+        <v>55</v>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="O56" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S56" s="3" t="n"/>
       <c r="T56" s="3" t="n"/>
     </row>
@@ -2492,14 +3372,30 @@
           <t>14:00</t>
         </is>
       </c>
-      <c r="D57" s="3" t="n"/>
+      <c r="D57" s="3" t="n">
+        <v>390.39</v>
+      </c>
       <c r="E57" s="3" t="n">
         <v>193.66</v>
       </c>
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="n"/>
-      <c r="M57" s="3" t="n"/>
-      <c r="O57" s="3" t="n"/>
+      <c r="L57" t="n">
+        <v>56</v>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S57" s="3" t="n"/>
       <c r="T57" s="3" t="n"/>
     </row>
@@ -2517,14 +3413,30 @@
           <t>14:15</t>
         </is>
       </c>
-      <c r="D58" s="3" t="n"/>
+      <c r="D58" s="3" t="n">
+        <v>263.48</v>
+      </c>
       <c r="E58" s="3" t="n">
         <v>193.66</v>
       </c>
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
-      <c r="M58" s="3" t="n"/>
-      <c r="O58" s="3" t="n"/>
+      <c r="L58" t="n">
+        <v>57</v>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S58" s="3" t="n"/>
       <c r="T58" s="3" t="n"/>
     </row>
@@ -2542,14 +3454,30 @@
           <t>14:30</t>
         </is>
       </c>
-      <c r="D59" s="3" t="n"/>
+      <c r="D59" s="3" t="n">
+        <v>263.48</v>
+      </c>
       <c r="E59" s="3" t="n">
         <v>462.51</v>
       </c>
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="n"/>
-      <c r="M59" s="3" t="n"/>
-      <c r="O59" s="3" t="n"/>
+      <c r="L59" t="n">
+        <v>58</v>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S59" s="3" t="n"/>
       <c r="T59" s="3" t="n"/>
     </row>
@@ -2567,14 +3495,30 @@
           <t>14:45</t>
         </is>
       </c>
-      <c r="D60" s="3" t="n"/>
+      <c r="D60" s="3" t="n">
+        <v>263.48</v>
+      </c>
       <c r="E60" s="3" t="n">
         <v>465.83</v>
       </c>
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
-      <c r="M60" s="3" t="n"/>
-      <c r="O60" s="3" t="n"/>
+      <c r="L60" t="n">
+        <v>59</v>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="O60" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S60" s="3" t="n"/>
       <c r="T60" s="3" t="n"/>
     </row>
@@ -2592,14 +3536,30 @@
           <t>15:00</t>
         </is>
       </c>
-      <c r="D61" s="3" t="n"/>
+      <c r="D61" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E61" s="3" t="n">
         <v>435</v>
       </c>
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
-      <c r="M61" s="3" t="n"/>
-      <c r="O61" s="3" t="n"/>
+      <c r="L61" t="n">
+        <v>60</v>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="n">
+        <v>98.19</v>
+      </c>
       <c r="S61" s="3" t="n"/>
       <c r="T61" s="3" t="n"/>
     </row>
@@ -2617,14 +3577,30 @@
           <t>15:15</t>
         </is>
       </c>
-      <c r="D62" s="3" t="n"/>
+      <c r="D62" s="3" t="n">
+        <v>422.32</v>
+      </c>
       <c r="E62" s="3" t="n">
         <v>494.04</v>
       </c>
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
-      <c r="M62" s="3" t="n"/>
-      <c r="O62" s="3" t="n"/>
+      <c r="L62" t="n">
+        <v>61</v>
+      </c>
+      <c r="M62" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="O62" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S62" s="3" t="n"/>
       <c r="T62" s="3" t="n"/>
     </row>
@@ -2642,14 +3618,30 @@
           <t>15:30</t>
         </is>
       </c>
-      <c r="D63" s="3" t="n"/>
+      <c r="D63" s="3" t="n">
+        <v>422.32</v>
+      </c>
       <c r="E63" s="3" t="n">
         <v>483.11</v>
       </c>
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="n"/>
-      <c r="M63" s="3" t="n"/>
-      <c r="O63" s="3" t="n"/>
+      <c r="L63" t="n">
+        <v>62</v>
+      </c>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="O63" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S63" s="3" t="n"/>
       <c r="T63" s="3" t="n"/>
     </row>
@@ -2667,14 +3659,30 @@
           <t>15:45</t>
         </is>
       </c>
-      <c r="D64" s="3" t="n"/>
+      <c r="D64" s="3" t="n">
+        <v>422.32</v>
+      </c>
       <c r="E64" s="3" t="n">
         <v>491.02</v>
       </c>
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
-      <c r="M64" s="3" t="n"/>
-      <c r="O64" s="3" t="n"/>
+      <c r="L64" t="n">
+        <v>63</v>
+      </c>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="O64" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S64" s="3" t="n"/>
       <c r="T64" s="3" t="n"/>
     </row>
@@ -2692,14 +3700,30 @@
           <t>16:00</t>
         </is>
       </c>
-      <c r="D65" s="3" t="n"/>
+      <c r="D65" s="3" t="n">
+        <v>433.7</v>
+      </c>
       <c r="E65" s="3" t="n">
         <v>438.54</v>
       </c>
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="n"/>
-      <c r="M65" s="3" t="n"/>
-      <c r="O65" s="3" t="n"/>
+      <c r="L65" t="n">
+        <v>64</v>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="O65" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S65" s="3" t="n"/>
       <c r="T65" s="3" t="n"/>
     </row>
@@ -2717,14 +3741,30 @@
           <t>16:15</t>
         </is>
       </c>
-      <c r="D66" s="3" t="n"/>
+      <c r="D66" s="3" t="n">
+        <v>450.72</v>
+      </c>
       <c r="E66" s="3" t="n">
         <v>491.02</v>
       </c>
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
-      <c r="M66" s="3" t="n"/>
-      <c r="O66" s="3" t="n"/>
+      <c r="L66" t="n">
+        <v>65</v>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="O66" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S66" s="3" t="n"/>
       <c r="T66" s="3" t="n"/>
     </row>
@@ -2742,14 +3782,30 @@
           <t>16:30</t>
         </is>
       </c>
-      <c r="D67" s="3" t="n"/>
+      <c r="D67" s="3" t="n">
+        <v>450.72</v>
+      </c>
       <c r="E67" s="3" t="n">
         <v>470</v>
       </c>
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
-      <c r="M67" s="3" t="n"/>
-      <c r="O67" s="3" t="n"/>
+      <c r="L67" t="n">
+        <v>66</v>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="O67" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S67" s="3" t="n"/>
       <c r="T67" s="3" t="n"/>
     </row>
@@ -2767,14 +3823,30 @@
           <t>16:45</t>
         </is>
       </c>
-      <c r="D68" s="3" t="n"/>
+      <c r="D68" s="3" t="n">
+        <v>450.72</v>
+      </c>
       <c r="E68" s="3" t="n">
         <v>483.2</v>
       </c>
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
-      <c r="M68" s="3" t="n"/>
-      <c r="O68" s="3" t="n"/>
+      <c r="L68" t="n">
+        <v>67</v>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="O68" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S68" s="3" t="n"/>
       <c r="T68" s="3" t="n"/>
     </row>
@@ -2792,14 +3864,30 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="D69" s="3" t="n"/>
+      <c r="D69" s="3" t="n">
+        <v>466.82</v>
+      </c>
       <c r="E69" s="3" t="n">
         <v>475</v>
       </c>
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
-      <c r="M69" s="3" t="n"/>
-      <c r="O69" s="3" t="n"/>
+      <c r="L69" t="n">
+        <v>68</v>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="O69" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S69" s="3" t="n"/>
       <c r="T69" s="3" t="n"/>
     </row>
@@ -2817,14 +3905,30 @@
           <t>17:15</t>
         </is>
       </c>
-      <c r="D70" s="3" t="n"/>
+      <c r="D70" s="3" t="n">
+        <v>475.69</v>
+      </c>
       <c r="E70" s="3" t="n">
         <v>470</v>
       </c>
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
-      <c r="M70" s="3" t="n"/>
-      <c r="O70" s="3" t="n"/>
+      <c r="L70" t="n">
+        <v>69</v>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="O70" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S70" s="3" t="n"/>
       <c r="T70" s="3" t="n"/>
     </row>
@@ -2842,14 +3946,30 @@
           <t>17:30</t>
         </is>
       </c>
-      <c r="D71" s="3" t="n"/>
+      <c r="D71" s="3" t="n">
+        <v>475.69</v>
+      </c>
       <c r="E71" s="3" t="n">
         <v>484.72</v>
       </c>
       <c r="H71" s="3" t="n"/>
       <c r="I71" s="3" t="n"/>
-      <c r="M71" s="3" t="n"/>
-      <c r="O71" s="3" t="n"/>
+      <c r="L71" t="n">
+        <v>70</v>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="O71" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S71" s="3" t="n"/>
       <c r="T71" s="3" t="n"/>
     </row>
@@ -2867,14 +3987,30 @@
           <t>17:45</t>
         </is>
       </c>
-      <c r="D72" s="3" t="n"/>
+      <c r="D72" s="3" t="n">
+        <v>475.69</v>
+      </c>
       <c r="E72" s="3" t="n">
         <v>486.94</v>
       </c>
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
-      <c r="M72" s="3" t="n"/>
-      <c r="O72" s="3" t="n"/>
+      <c r="L72" t="n">
+        <v>71</v>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="O72" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S72" s="3" t="n"/>
       <c r="T72" s="3" t="n"/>
     </row>
@@ -2892,14 +4028,30 @@
           <t>18:00</t>
         </is>
       </c>
-      <c r="D73" s="3" t="n"/>
+      <c r="D73" s="3" t="n">
+        <v>475.69</v>
+      </c>
       <c r="E73" s="3" t="n">
         <v>491.14</v>
       </c>
       <c r="H73" s="3" t="n"/>
       <c r="I73" s="3" t="n"/>
-      <c r="M73" s="3" t="n"/>
-      <c r="O73" s="3" t="n"/>
+      <c r="L73" t="n">
+        <v>72</v>
+      </c>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="O73" s="3" t="n">
+        <v>280.3</v>
+      </c>
       <c r="S73" s="3" t="n"/>
       <c r="T73" s="3" t="n"/>
     </row>
@@ -2917,14 +4069,30 @@
           <t>18:15</t>
         </is>
       </c>
-      <c r="D74" s="3" t="n"/>
+      <c r="D74" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E74" s="3" t="n">
         <v>483.11</v>
       </c>
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
-      <c r="M74" s="3" t="n"/>
-      <c r="O74" s="3" t="n"/>
+      <c r="L74" t="n">
+        <v>73</v>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="O74" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S74" s="3" t="n"/>
       <c r="T74" s="3" t="n"/>
     </row>
@@ -2942,14 +4110,30 @@
           <t>18:30</t>
         </is>
       </c>
-      <c r="D75" s="3" t="n"/>
+      <c r="D75" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E75" s="3" t="n">
         <v>471.52</v>
       </c>
       <c r="H75" s="3" t="n"/>
       <c r="I75" s="3" t="n"/>
-      <c r="M75" s="3" t="n"/>
-      <c r="O75" s="3" t="n"/>
+      <c r="L75" t="n">
+        <v>74</v>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="O75" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S75" s="3" t="n"/>
       <c r="T75" s="3" t="n"/>
     </row>
@@ -2967,14 +4151,30 @@
           <t>18:45</t>
         </is>
       </c>
-      <c r="D76" s="3" t="n"/>
+      <c r="D76" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E76" s="3" t="n">
         <v>471.89</v>
       </c>
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
-      <c r="M76" s="3" t="n"/>
-      <c r="O76" s="3" t="n"/>
+      <c r="L76" t="n">
+        <v>75</v>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="O76" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S76" s="3" t="n"/>
       <c r="T76" s="3" t="n"/>
     </row>
@@ -2992,14 +4192,30 @@
           <t>19:00</t>
         </is>
       </c>
-      <c r="D77" s="3" t="n"/>
+      <c r="D77" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E77" s="3" t="n">
         <v>470.02</v>
       </c>
       <c r="H77" s="3" t="n"/>
       <c r="I77" s="3" t="n"/>
-      <c r="M77" s="3" t="n"/>
-      <c r="O77" s="3" t="n"/>
+      <c r="L77" t="n">
+        <v>76</v>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="n">
+        <v>444.2</v>
+      </c>
       <c r="S77" s="3" t="n"/>
       <c r="T77" s="3" t="n"/>
     </row>
@@ -3017,14 +4233,30 @@
           <t>19:15</t>
         </is>
       </c>
-      <c r="D78" s="3" t="n"/>
+      <c r="D78" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E78" s="3" t="n">
         <v>473.6</v>
       </c>
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
-      <c r="M78" s="3" t="n"/>
-      <c r="O78" s="3" t="n"/>
+      <c r="L78" t="n">
+        <v>77</v>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="O78" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S78" s="3" t="n"/>
       <c r="T78" s="3" t="n"/>
     </row>
@@ -3042,14 +4274,30 @@
           <t>19:30</t>
         </is>
       </c>
-      <c r="D79" s="3" t="n"/>
+      <c r="D79" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E79" s="3" t="n">
         <v>478.29</v>
       </c>
       <c r="H79" s="3" t="n"/>
       <c r="I79" s="3" t="n"/>
-      <c r="M79" s="3" t="n"/>
-      <c r="O79" s="3" t="n"/>
+      <c r="L79" t="n">
+        <v>78</v>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="O79" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S79" s="3" t="n"/>
       <c r="T79" s="3" t="n"/>
     </row>
@@ -3067,14 +4315,30 @@
           <t>19:45</t>
         </is>
       </c>
-      <c r="D80" s="3" t="n"/>
+      <c r="D80" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E80" s="3" t="n">
         <v>473.22</v>
       </c>
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
-      <c r="M80" s="3" t="n"/>
-      <c r="O80" s="3" t="n"/>
+      <c r="L80" t="n">
+        <v>79</v>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="O80" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S80" s="3" t="n"/>
       <c r="T80" s="3" t="n"/>
     </row>
@@ -3092,14 +4356,30 @@
           <t>20:00</t>
         </is>
       </c>
-      <c r="D81" s="3" t="n"/>
+      <c r="D81" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E81" s="3" t="n">
         <v>466.55</v>
       </c>
       <c r="H81" s="3" t="n"/>
       <c r="I81" s="3" t="n"/>
-      <c r="M81" s="3" t="n"/>
-      <c r="O81" s="3" t="n"/>
+      <c r="L81" t="n">
+        <v>80</v>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="O81" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S81" s="3" t="n"/>
       <c r="T81" s="3" t="n"/>
     </row>
@@ -3117,14 +4397,30 @@
           <t>20:15</t>
         </is>
       </c>
-      <c r="D82" s="3" t="n"/>
+      <c r="D82" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E82" s="3" t="n">
         <v>488.14</v>
       </c>
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
-      <c r="M82" s="3" t="n"/>
-      <c r="O82" s="3" t="n"/>
+      <c r="L82" t="n">
+        <v>81</v>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="O82" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S82" s="3" t="n"/>
       <c r="T82" s="3" t="n"/>
     </row>
@@ -3142,14 +4438,30 @@
           <t>20:30</t>
         </is>
       </c>
-      <c r="D83" s="3" t="n"/>
+      <c r="D83" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E83" s="3" t="n">
         <v>492.16</v>
       </c>
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
-      <c r="M83" s="3" t="n"/>
-      <c r="O83" s="3" t="n"/>
+      <c r="L83" t="n">
+        <v>82</v>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="O83" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S83" s="3" t="n"/>
       <c r="T83" s="3" t="n"/>
     </row>
@@ -3167,14 +4479,30 @@
           <t>20:45</t>
         </is>
       </c>
-      <c r="D84" s="3" t="n"/>
+      <c r="D84" s="3" t="n">
+        <v>409.48</v>
+      </c>
       <c r="E84" s="3" t="n">
         <v>494.44</v>
       </c>
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
-      <c r="M84" s="3" t="n"/>
-      <c r="O84" s="3" t="n"/>
+      <c r="L84" t="n">
+        <v>83</v>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S84" s="3" t="n"/>
       <c r="T84" s="3" t="n"/>
     </row>
@@ -3192,14 +4520,30 @@
           <t>21:00</t>
         </is>
       </c>
-      <c r="D85" s="3" t="n"/>
+      <c r="D85" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E85" s="3" t="n">
         <v>498.17</v>
       </c>
       <c r="H85" s="3" t="n"/>
       <c r="I85" s="3" t="n"/>
-      <c r="M85" s="3" t="n"/>
-      <c r="O85" s="3" t="n"/>
+      <c r="L85" t="n">
+        <v>84</v>
+      </c>
+      <c r="M85" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S85" s="3" t="n"/>
       <c r="T85" s="3" t="n"/>
     </row>
@@ -3217,14 +4561,30 @@
           <t>21:15</t>
         </is>
       </c>
-      <c r="D86" s="3" t="n"/>
+      <c r="D86" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E86" s="3" t="n">
         <v>495.52</v>
       </c>
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
-      <c r="M86" s="3" t="n"/>
-      <c r="O86" s="3" t="n"/>
+      <c r="L86" t="n">
+        <v>85</v>
+      </c>
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="O86" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S86" s="3" t="n"/>
       <c r="T86" s="3" t="n"/>
     </row>
@@ -3242,14 +4602,30 @@
           <t>21:30</t>
         </is>
       </c>
-      <c r="D87" s="3" t="n"/>
+      <c r="D87" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E87" s="3" t="n">
         <v>488.89</v>
       </c>
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="n"/>
-      <c r="M87" s="3" t="n"/>
-      <c r="O87" s="3" t="n"/>
+      <c r="L87" t="n">
+        <v>86</v>
+      </c>
+      <c r="M87" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="O87" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S87" s="3" t="n"/>
       <c r="T87" s="3" t="n"/>
     </row>
@@ -3267,14 +4643,30 @@
           <t>21:45</t>
         </is>
       </c>
-      <c r="D88" s="3" t="n"/>
+      <c r="D88" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E88" s="3" t="n">
         <v>474.02</v>
       </c>
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
-      <c r="M88" s="3" t="n"/>
-      <c r="O88" s="3" t="n"/>
+      <c r="L88" t="n">
+        <v>87</v>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="O88" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S88" s="3" t="n"/>
       <c r="T88" s="3" t="n"/>
     </row>
@@ -3292,14 +4684,30 @@
           <t>22:00</t>
         </is>
       </c>
-      <c r="D89" s="3" t="n"/>
+      <c r="D89" s="3" t="n">
+        <v>433.7</v>
+      </c>
       <c r="E89" s="3" t="n">
         <v>470</v>
       </c>
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="n"/>
-      <c r="M89" s="3" t="n"/>
-      <c r="O89" s="3" t="n"/>
+      <c r="L89" t="n">
+        <v>88</v>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="n">
+        <v>437.1</v>
+      </c>
       <c r="S89" s="3" t="n"/>
       <c r="T89" s="3" t="n"/>
     </row>
@@ -3317,14 +4725,30 @@
           <t>22:15</t>
         </is>
       </c>
-      <c r="D90" s="3" t="n"/>
+      <c r="D90" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E90" s="3" t="n">
         <v>460.82</v>
       </c>
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
-      <c r="M90" s="3" t="n"/>
-      <c r="O90" s="3" t="n"/>
+      <c r="L90" t="n">
+        <v>89</v>
+      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="O90" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S90" s="3" t="n"/>
       <c r="T90" s="3" t="n"/>
     </row>
@@ -3342,14 +4766,30 @@
           <t>22:30</t>
         </is>
       </c>
-      <c r="D91" s="3" t="n"/>
+      <c r="D91" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E91" s="3" t="n">
         <v>467.89</v>
       </c>
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="n"/>
-      <c r="M91" s="3" t="n"/>
-      <c r="O91" s="3" t="n"/>
+      <c r="L91" t="n">
+        <v>90</v>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="O91" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S91" s="3" t="n"/>
       <c r="T91" s="3" t="n"/>
     </row>
@@ -3367,14 +4807,30 @@
           <t>22:45</t>
         </is>
       </c>
-      <c r="D92" s="3" t="n"/>
+      <c r="D92" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E92" s="3" t="n">
         <v>109.9</v>
       </c>
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
-      <c r="M92" s="3" t="n"/>
-      <c r="O92" s="3" t="n"/>
+      <c r="L92" t="n">
+        <v>91</v>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="O92" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S92" s="3" t="n"/>
       <c r="T92" s="3" t="n"/>
     </row>
@@ -3392,13 +4848,29 @@
           <t>23:00</t>
         </is>
       </c>
-      <c r="D93" s="3" t="n"/>
+      <c r="D93" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E93" s="3" t="n">
         <v>435.54</v>
       </c>
       <c r="I93" s="3" t="n"/>
-      <c r="M93" s="3" t="n"/>
-      <c r="O93" s="3" t="n"/>
+      <c r="L93" t="n">
+        <v>92</v>
+      </c>
+      <c r="M93" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="O93" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S93" s="3" t="n"/>
       <c r="T93" s="3" t="n"/>
     </row>
@@ -3416,13 +4888,29 @@
           <t>23:15</t>
         </is>
       </c>
-      <c r="D94" s="3" t="n"/>
+      <c r="D94" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E94" s="3" t="n">
         <v>456.07</v>
       </c>
       <c r="I94" s="3" t="n"/>
-      <c r="M94" s="3" t="n"/>
-      <c r="O94" s="3" t="n"/>
+      <c r="L94" t="n">
+        <v>93</v>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="O94" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S94" s="3" t="n"/>
       <c r="T94" s="3" t="n"/>
     </row>
@@ -3440,13 +4928,29 @@
           <t>23:30</t>
         </is>
       </c>
-      <c r="D95" s="3" t="n"/>
+      <c r="D95" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E95" s="3" t="n">
         <v>452.22</v>
       </c>
       <c r="I95" s="3" t="n"/>
-      <c r="M95" s="3" t="n"/>
-      <c r="O95" s="3" t="n"/>
+      <c r="L95" t="n">
+        <v>94</v>
+      </c>
+      <c r="M95" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="O95" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S95" s="3" t="n"/>
       <c r="T95" s="3" t="n"/>
     </row>
@@ -3464,13 +4968,29 @@
           <t>23:45</t>
         </is>
       </c>
-      <c r="D96" s="3" t="n"/>
+      <c r="D96" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E96" s="3" t="n">
         <v>441.17</v>
       </c>
       <c r="I96" s="3" t="n"/>
-      <c r="M96" s="3" t="n"/>
-      <c r="O96" s="3" t="n"/>
+      <c r="L96" t="n">
+        <v>95</v>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="O96" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S96" s="3" t="n"/>
       <c r="T96" s="3" t="n"/>
     </row>
@@ -3488,14 +5008,30 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="D97" s="3" t="n"/>
+      <c r="D97" s="3" t="n">
+        <v>433.64</v>
+      </c>
       <c r="E97" s="3" t="n">
         <v>442.35</v>
       </c>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
-      <c r="M97" s="3" t="n"/>
-      <c r="O97" s="3" t="n"/>
+      <c r="L97" t="n">
+        <v>96</v>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>20261023</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="n">
+        <v>424.45</v>
+      </c>
       <c r="S97" s="3" t="n"/>
       <c r="T97" s="3" t="n"/>
     </row>
@@ -3577,8 +5113,27 @@
       </c>
     </row>
     <row r="2">
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>11921.936</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>317.045</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3602,8 +5157,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>11887.836</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>315.09</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3627,8 +5201,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>14795.839</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>281.525</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3652,8 +5245,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>13010.85</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>164.943</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3677,8 +5289,27 @@
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>12251.947</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>214.405</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3702,8 +5333,27 @@
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>12613.756</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>310.538</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3727,8 +5377,27 @@
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>14751.349</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>455.483</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3752,8 +5421,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>15304.06</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>275.043</v>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3777,8 +5465,27 @@
       </c>
     </row>
     <row r="10">
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>14399.475</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>60.355</v>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3802,8 +5509,27 @@
       </c>
     </row>
     <row r="11">
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>14064.668</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>148.47</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3827,8 +5553,27 @@
       </c>
     </row>
     <row r="12">
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>14570.126</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>156.32</v>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3852,8 +5597,27 @@
       </c>
     </row>
     <row r="13">
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>15552.088</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>220.32</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3877,8 +5641,27 @@
       </c>
     </row>
     <row r="14">
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>15000.753</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>212.038</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3902,8 +5685,27 @@
       </c>
     </row>
     <row r="15">
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>16201.801</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>322.728</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3927,8 +5729,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>16212.132</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>389.25</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3952,8 +5773,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>15533.14</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>476.678</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -3977,8 +5817,27 @@
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>15437.802</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>479.805</v>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4002,8 +5861,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>15081.26</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>483.2</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4027,8 +5905,27 @@
       </c>
     </row>
     <row r="20">
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>13492.461</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>474.135</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4052,8 +5949,27 @@
       </c>
     </row>
     <row r="21">
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>12824.555</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>472.915</v>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4077,8 +5993,27 @@
       </c>
     </row>
     <row r="22">
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>13186.298</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>493.228</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4102,8 +6037,27 @@
       </c>
     </row>
     <row r="23">
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>13485.187</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>482.108</v>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4127,8 +6081,27 @@
       </c>
     </row>
     <row r="24">
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>11817.839</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>368.538</v>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -4152,8 +6125,27 @@
       </c>
     </row>
     <row r="25">
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>10693.977</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>447.953</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -15295,7 +17287,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>现货日前交易价格曲线</t>
+          <t>现货实时交易价格曲线</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -15308,46 +17300,46 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>非市场化机组总出力</t>
+          <t>现货日前交易价格曲线</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>新能源实际发电曲线</t>
+          <t>非市场化机组总出力</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>96</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>实际系统负荷</t>
+          <t>新能源实际发电曲线</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>96</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>省间联络线输电情况</t>
+          <t>实际系统负荷</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -15360,24 +17352,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>各时段各类电源电量</t>
+          <t>省间联络线输电情况</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>960</v>
+        <v>96</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>各时段各类电源的开机台数</t>
+          <t>各时段各类电源电量</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>768</v>
+        <v>960</v>
       </c>
       <c r="C8" t="n">
         <v>5</v>
@@ -15386,18 +17378,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>各时段各类电源的开机台数</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>768</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>实时储能充电计划及电价</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>96</v>
       </c>
-      <c r="C9" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11"/>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>日前储能充电计划及电价</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>96</v>
+      </c>
+      <c r="C11" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>